<commit_message>
Objective ratings: one published rule for every report (value against the S&P 500 on the same assumptions), neutral closing text, scenario models now count cash flow before 2030, calibration on the About page, primary sources and labelled estimates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HR3LbNEqqh1NJpsKSu2JUT
</commit_message>
<xml_diff>
--- a/data/models/amd.xlsx
+++ b/data/models/amd.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="46">
   <si>
     <t xml:space="preserve">LDB FINANCE</t>
   </si>
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Advanced Micro Devices (AMD)</t>
   </si>
   <si>
-    <t xml:space="preserve">Scenario model: 2030 earning power, capitalised and discounted back four years  ·  Inputs in blue can be changed; everything else recalculates.</t>
+    <t xml:space="preserve">Scenario model: 2030 earning power, capitalised and discounted back four years, plus cash flow along the way  ·  Inputs in blue can be changed; everything else recalculates.</t>
   </si>
   <si>
     <t xml:space="preserve">SCENARIOS</t>
@@ -116,6 +116,18 @@
     <t xml:space="preserve">Shares by 2030 (billions)</t>
   </si>
   <si>
+    <t xml:space="preserve">Free cash flow this year ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating cash flow less capital spending, last twelve months</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free cash flow in 2030, share of after-tax profit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The rest is reinvested</t>
+  </si>
+  <si>
     <t xml:space="preserve">VALUE</t>
   </si>
   <si>
@@ -128,7 +140,25 @@
     <t xml:space="preserve">Value today ($B)</t>
   </si>
   <si>
-    <t xml:space="preserve">Plus net cash: equity value ($B)</t>
+    <t xml:space="preserve">Free cash flow in 2030 ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free cash flow, year 1 ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free cash flow, year 2 ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free cash flow, year 3 ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Free cash flow, year 4 ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Present value of free cash flow, years 1-4 ($B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plus cash flow and net cash: equity value ($B)</t>
   </si>
 </sst>
 </file>
@@ -752,16 +782,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="10" t="n">
-        <f aca="false">Model!B23</f>
-        <v>128.225602251955</v>
+        <f aca="false">Model!B31</f>
+        <v>147.876882172937</v>
       </c>
       <c r="C8" s="10" t="n">
-        <f aca="false">Model!C23</f>
-        <v>319.287051212385</v>
+        <f aca="false">Model!C31</f>
+        <v>353.402979471444</v>
       </c>
       <c r="D8" s="10" t="n">
-        <f aca="false">Model!D23</f>
-        <v>591.235828929786</v>
+        <f aca="false">Model!D31</f>
+        <v>641.07420103458</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -784,7 +814,7 @@
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">SUMPRODUCT(B8:D8,B9:D9)</f>
-        <v>339.508883401628</v>
+        <v>373.939260537601</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -801,7 +831,7 @@
       </c>
       <c r="C12" s="15" t="n">
         <f aca="false">C10/C11-1</f>
-        <v>-0.385748872120372</v>
+        <v>-0.323456251741205</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -830,8 +860,8 @@
         <v>0.1</v>
       </c>
       <c r="C16" s="18" t="n">
-        <f aca="false">(Model!$C$20/(1+B16)^Model!$C$13+Model!$C$14)/Model!$C$15</f>
-        <v>342.737893586504</v>
+        <f aca="false">(Model!$C$22/(1+B16)^Model!$C$13+Model!$C$25/(1+B16)^1+Model!$C$26/(1+B16)^2+Model!$C$27/(1+B16)^3+Model!$C$28/(1+B16)^4+Model!$C$14)/Model!$C$15</f>
+        <v>378.53914805455</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -840,8 +870,8 @@
         <v>0.11</v>
       </c>
       <c r="C17" s="18" t="n">
-        <f aca="false">(Model!$C$20/(1+B17)^Model!$C$13+Model!$C$14)/Model!$C$15</f>
-        <v>330.748418484094</v>
+        <f aca="false">(Model!$C$22/(1+B17)^Model!$C$13+Model!$C$25/(1+B17)^1+Model!$C$26/(1+B17)^2+Model!$C$27/(1+B17)^3+Model!$C$28/(1+B17)^4+Model!$C$14)/Model!$C$15</f>
+        <v>365.691356967428</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -850,8 +880,8 @@
         <v>0.12</v>
       </c>
       <c r="C18" s="18" t="n">
-        <f aca="false">(Model!$C$20/(1+B18)^Model!$C$13+Model!$C$14)/Model!$C$15</f>
-        <v>319.287051212385</v>
+        <f aca="false">(Model!$C$22/(1+B18)^Model!$C$13+Model!$C$25/(1+B18)^1+Model!$C$26/(1+B18)^2+Model!$C$27/(1+B18)^3+Model!$C$28/(1+B18)^4+Model!$C$14)/Model!$C$15</f>
+        <v>353.402979471444</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -860,8 +890,8 @@
         <v>0.13</v>
       </c>
       <c r="C19" s="18" t="n">
-        <f aca="false">(Model!$C$20/(1+B19)^Model!$C$13+Model!$C$14)/Model!$C$15</f>
-        <v>308.326121791692</v>
+        <f aca="false">(Model!$C$22/(1+B19)^Model!$C$13+Model!$C$25/(1+B19)^1+Model!$C$26/(1+B19)^2+Model!$C$27/(1+B19)^3+Model!$C$28/(1+B19)^4+Model!$C$14)/Model!$C$15</f>
+        <v>341.644882048515</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -870,8 +900,8 @@
         <v>0.14</v>
       </c>
       <c r="C20" s="18" t="n">
-        <f aca="false">(Model!$C$20/(1+B20)^Model!$C$13+Model!$C$14)/Model!$C$15</f>
-        <v>297.839636951531</v>
+        <f aca="false">(Model!$C$22/(1+B20)^Model!$C$13+Model!$C$25/(1+B20)^1+Model!$C$26/(1+B20)^2+Model!$C$27/(1+B20)^3+Model!$C$28/(1+B20)^4+Model!$C$14)/Model!$C$15</f>
+        <v>330.389689997187</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -919,7 +949,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="48"/>
@@ -1097,110 +1127,246 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-    </row>
-    <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7"/>
-      <c r="B18" s="8" t="s">
+      <c r="B16" s="20" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="C16" s="20" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="D16" s="20" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="E16" s="19" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C17" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E17" s="19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+    </row>
+    <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="7"/>
+      <c r="B20" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C20" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D20" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="24" t="n">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="24" t="n">
         <f aca="false">B8*B9*(1-B10)</f>
         <v>17.38</v>
       </c>
-      <c r="C19" s="24" t="n">
+      <c r="C21" s="24" t="n">
         <f aca="false">C8*C9*(1-C10)</f>
         <v>35.55</v>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D21" s="24" t="n">
         <f aca="false">D8*D9*(1-D10)</f>
         <v>55.3</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="24" t="n">
-        <f aca="false">B19*B11</f>
-        <v>347.6</v>
-      </c>
-      <c r="C20" s="24" t="n">
-        <f aca="false">C19*C11</f>
-        <v>888.75</v>
-      </c>
-      <c r="D20" s="24" t="n">
-        <f aca="false">D19*D11</f>
-        <v>1659</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="B21" s="24" t="n">
-        <f aca="false">B20/(1+B12)^B13</f>
-        <v>220.906084053519</v>
-      </c>
-      <c r="C21" s="24" t="n">
-        <f aca="false">C20/(1+C12)^C13</f>
-        <v>564.816692182294</v>
-      </c>
-      <c r="D21" s="24" t="n">
-        <f aca="false">D20/(1+D12)^D13</f>
-        <v>1054.32449207362</v>
-      </c>
-    </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B22" s="24" t="n">
-        <f aca="false">B21+B14</f>
-        <v>230.806084053519</v>
+        <f aca="false">B21*B11</f>
+        <v>347.6</v>
       </c>
       <c r="C22" s="24" t="n">
-        <f aca="false">C21+C14</f>
-        <v>574.716692182294</v>
+        <f aca="false">C21*C11</f>
+        <v>888.75</v>
       </c>
       <c r="D22" s="24" t="n">
-        <f aca="false">D21+D14</f>
-        <v>1064.22449207362</v>
+        <f aca="false">D21*D11</f>
+        <v>1659</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="24" t="n">
+        <f aca="false">B22/(1+B12)^B13</f>
+        <v>220.906084053519</v>
+      </c>
+      <c r="C23" s="24" t="n">
+        <f aca="false">C22/(1+C12)^C13</f>
+        <v>564.816692182294</v>
+      </c>
+      <c r="D23" s="24" t="n">
+        <f aca="false">D22/(1+D12)^D13</f>
+        <v>1054.32449207362</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" s="24" t="n">
+        <f aca="false">B21*B17</f>
+        <v>13.904</v>
+      </c>
+      <c r="C24" s="24" t="n">
+        <f aca="false">C21*C17</f>
+        <v>28.44</v>
+      </c>
+      <c r="D24" s="24" t="n">
+        <f aca="false">D21*D17</f>
+        <v>44.24</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="24" t="n">
+        <f aca="false">B16+(B24-B16)*1/B13</f>
+        <v>9.776</v>
+      </c>
+      <c r="C25" s="24" t="n">
+        <f aca="false">C16+(C24-C16)*1/C13</f>
+        <v>13.41</v>
+      </c>
+      <c r="D25" s="24" t="n">
+        <f aca="false">D16+(D24-D16)*1/D13</f>
+        <v>17.36</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B26" s="24" t="n">
+        <f aca="false">B16+(B24-B16)*2/B13</f>
+        <v>11.152</v>
+      </c>
+      <c r="C26" s="24" t="n">
+        <f aca="false">C16+(C24-C16)*2/C13</f>
+        <v>18.42</v>
+      </c>
+      <c r="D26" s="24" t="n">
+        <f aca="false">D16+(D24-D16)*2/D13</f>
+        <v>26.32</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B27" s="24" t="n">
+        <f aca="false">B16+(B24-B16)*3/B13</f>
+        <v>12.528</v>
+      </c>
+      <c r="C27" s="24" t="n">
+        <f aca="false">C16+(C24-C16)*3/C13</f>
+        <v>23.43</v>
+      </c>
+      <c r="D27" s="24" t="n">
+        <f aca="false">D16+(D24-D16)*3/D13</f>
+        <v>35.28</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B28" s="24" t="n">
+        <f aca="false">B16+(B24-B16)*4/B13</f>
+        <v>13.904</v>
+      </c>
+      <c r="C28" s="24" t="n">
+        <f aca="false">C16+(C24-C16)*4/C13</f>
+        <v>28.44</v>
+      </c>
+      <c r="D28" s="24" t="n">
+        <f aca="false">D16+(D24-D16)*4/D13</f>
+        <v>44.24</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="24" t="n">
+        <f aca="false">B25/(1+B12)^1+B26/(1+B12)^2+B27/(1+B12)^3+B28/(1+B12)^4</f>
+        <v>35.3723038577676</v>
+      </c>
+      <c r="C29" s="24" t="n">
+        <f aca="false">C25/(1+C12)^1+C26/(1+C12)^2+C27/(1+C12)^3+C28/(1+C12)^4</f>
+        <v>61.4086708663057</v>
+      </c>
+      <c r="D29" s="24" t="n">
+        <f aca="false">D25/(1+D12)^1+D26/(1+D12)^2+D27/(1+D12)^3+D28/(1+D12)^4</f>
+        <v>89.7090697886297</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B30" s="24" t="n">
+        <f aca="false">B23+B29+B14</f>
+        <v>266.178387911287</v>
+      </c>
+      <c r="C30" s="24" t="n">
+        <f aca="false">C23+C29+C14</f>
+        <v>636.125363048599</v>
+      </c>
+      <c r="D30" s="24" t="n">
+        <f aca="false">D23+D29+D14</f>
+        <v>1153.93356186224</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B23" s="13" t="n">
-        <f aca="false">B22/B15</f>
-        <v>128.225602251955</v>
-      </c>
-      <c r="C23" s="13" t="n">
-        <f aca="false">C22/C15</f>
-        <v>319.287051212385</v>
-      </c>
-      <c r="D23" s="13" t="n">
-        <f aca="false">D22/D15</f>
-        <v>591.235828929786</v>
+      <c r="B31" s="13" t="n">
+        <f aca="false">B30/B15</f>
+        <v>147.876882172937</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <f aca="false">C30/C15</f>
+        <v>353.402979471444</v>
+      </c>
+      <c r="D31" s="13" t="n">
+        <f aca="false">D30/D15</f>
+        <v>641.07420103458</v>
       </c>
     </row>
   </sheetData>

</xml_diff>